<commit_message>
Update ablation analysis and vulnerability categories
</commit_message>
<xml_diff>
--- a/outputs/midhili/Ablation_Kappa_Comparison/Midhili_Ablation_Kappa_Comparison.xlsx
+++ b/outputs/midhili/Ablation_Kappa_Comparison/Midhili_Ablation_Kappa_Comparison.xlsx
@@ -903,20 +903,20 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>5 / 60</t>
+          <t>4 / 12</t>
         </is>
       </c>
       <c r="G8" s="4" t="n">
-        <v>0.1665638494756323</v>
+        <v>0.1850989522700814</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>27.55102040816326</v>
+        <v>17.3469387755102</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>32.6530612244898</v>
+        <v>43.87755102040816</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>39.79591836734694</v>
+        <v>38.77551020408163</v>
       </c>
     </row>
     <row r="9">
@@ -945,20 +945,20 @@
       </c>
       <c r="F9" s="7" t="inlineStr">
         <is>
-          <t>5 / 60</t>
+          <t>4 / 12</t>
         </is>
       </c>
       <c r="G9" s="4" t="n">
-        <v>0.2600766639563248</v>
+        <v>0.2357019064124782</v>
       </c>
       <c r="H9" s="8" t="n">
-        <v>22.44897959183674</v>
+        <v>8.163265306122449</v>
       </c>
       <c r="I9" s="8" t="n">
-        <v>59.18367346938776</v>
+        <v>64.28571428571429</v>
       </c>
       <c r="J9" s="8" t="n">
-        <v>18.36734693877551</v>
+        <v>27.55102040816326</v>
       </c>
     </row>
     <row r="10">
@@ -987,20 +987,20 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>5 / 60</t>
+          <t>4 / 12</t>
         </is>
       </c>
       <c r="G10" s="4" t="n">
-        <v>0.1699668078287743</v>
+        <v>0.01525210837968782</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>25.51020408163265</v>
+        <v>12.24489795918367</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>48.97959183673469</v>
+        <v>40.81632653061224</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>25.51020408163265</v>
+        <v>46.93877551020408</v>
       </c>
     </row>
     <row r="11">
@@ -1369,16 +1369,16 @@
         </is>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.1745722138487455</v>
+        <v>0.0495781508219536</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>4.081632653061225</v>
+        <v>10.20408163265306</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>63.26530612244898</v>
+        <v>43.87755102040816</v>
       </c>
       <c r="J19" s="8" t="n">
-        <v>32.6530612244898</v>
+        <v>45.91836734693878</v>
       </c>
     </row>
     <row r="20">
@@ -1747,16 +1747,16 @@
         </is>
       </c>
       <c r="G28" s="4" t="n">
-        <v>0.1389564747228981</v>
+        <v>0.09841092835238363</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>34.69387755102041</v>
+        <v>38.77551020408163</v>
       </c>
       <c r="I28" s="5" t="n">
-        <v>42.85714285714285</v>
+        <v>36.73469387755102</v>
       </c>
       <c r="J28" s="5" t="n">
-        <v>22.44897959183674</v>
+        <v>24.48979591836735</v>
       </c>
     </row>
     <row r="29">
@@ -2125,16 +2125,16 @@
         </is>
       </c>
       <c r="G37" s="4" t="n">
-        <v>0.07470147181338516</v>
+        <v>0.04499856692462023</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>30.61224489795918</v>
+        <v>40.81632653061224</v>
       </c>
       <c r="I37" s="8" t="n">
-        <v>47.95918367346938</v>
+        <v>32.6530612244898</v>
       </c>
       <c r="J37" s="8" t="n">
-        <v>21.42857142857143</v>
+        <v>26.53061224489796</v>
       </c>
     </row>
   </sheetData>
@@ -2426,20 +2426,20 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>5 / 60</t>
+          <t>4 / 12</t>
         </is>
       </c>
       <c r="E11" s="4" t="n">
-        <v>0.1665638494756323</v>
+        <v>0.1850989522700814</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>27.55102040816326</v>
+        <v>17.3469387755102</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>32.6530612244898</v>
+        <v>43.87755102040816</v>
       </c>
       <c r="H11" s="8" t="n">
-        <v>39.79591836734694</v>
+        <v>38.77551020408163</v>
       </c>
     </row>
     <row r="12">
@@ -2458,20 +2458,20 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>5 / 60</t>
+          <t>4 / 12</t>
         </is>
       </c>
       <c r="E12" s="4" t="n">
-        <v>0.2600766639563248</v>
+        <v>0.2357019064124782</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>22.44897959183674</v>
+        <v>8.163265306122449</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>59.18367346938776</v>
+        <v>64.28571428571429</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>18.36734693877551</v>
+        <v>27.55102040816326</v>
       </c>
     </row>
     <row r="13">
@@ -2490,20 +2490,20 @@
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>5 / 60</t>
+          <t>4 / 12</t>
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.1699668078287743</v>
+        <v>0.01525210837968782</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>25.51020408163265</v>
+        <v>12.24489795918367</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>48.97959183673469</v>
+        <v>40.81632653061224</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>25.51020408163265</v>
+        <v>46.93877551020408</v>
       </c>
     </row>
   </sheetData>
@@ -2867,16 +2867,16 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.1745722138487455</v>
+        <v>0.0495781508219536</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>4.081632653061225</v>
+        <v>10.20408163265306</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>63.26530612244898</v>
+        <v>43.87755102040816</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>32.6530612244898</v>
+        <v>45.91836734693878</v>
       </c>
     </row>
   </sheetData>
@@ -3240,16 +3240,16 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.1389564747228981</v>
+        <v>0.09841092835238363</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>34.69387755102041</v>
+        <v>38.77551020408163</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>42.85714285714285</v>
+        <v>36.73469387755102</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>22.44897959183674</v>
+        <v>24.48979591836735</v>
       </c>
     </row>
   </sheetData>
@@ -3613,16 +3613,16 @@
         </is>
       </c>
       <c r="E13" s="4" t="n">
-        <v>0.07470147181338516</v>
+        <v>0.04499856692462023</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>30.61224489795918</v>
+        <v>40.81632653061224</v>
       </c>
       <c r="G13" s="8" t="n">
-        <v>47.95918367346938</v>
+        <v>32.6530612244898</v>
       </c>
       <c r="H13" s="8" t="n">
-        <v>21.42857142857143</v>
+        <v>26.53061224489796</v>
       </c>
     </row>
   </sheetData>
@@ -3989,22 +3989,22 @@
         </is>
       </c>
       <c r="D8" s="15" t="n">
-        <v>0.1665638494756323</v>
+        <v>0.1850989522700814</v>
       </c>
       <c r="E8" s="15" t="n">
-        <v>27.55102040816326</v>
+        <v>17.3469387755102</v>
       </c>
       <c r="F8" s="15" t="n">
-        <v>32.6530612244898</v>
+        <v>43.87755102040816</v>
       </c>
       <c r="G8" s="15" t="n">
-        <v>60.20408163265306</v>
+        <v>61.22448979591837</v>
       </c>
       <c r="H8" s="15" t="n">
-        <v>60.20408163265306</v>
+        <v>61.22448979591837</v>
       </c>
       <c r="I8" s="15" t="n">
-        <v>39.79591836734694</v>
+        <v>38.77551020408163</v>
       </c>
       <c r="J8" s="15" t="n">
         <v>100</v>
@@ -4032,22 +4032,22 @@
         </is>
       </c>
       <c r="D9" s="15" t="n">
-        <v>0.2600766639563248</v>
+        <v>0.2357019064124782</v>
       </c>
       <c r="E9" s="15" t="n">
-        <v>22.44897959183674</v>
+        <v>8.163265306122449</v>
       </c>
       <c r="F9" s="15" t="n">
-        <v>59.18367346938776</v>
+        <v>64.28571428571429</v>
       </c>
       <c r="G9" s="15" t="n">
-        <v>81.63265306122449</v>
+        <v>72.44897959183673</v>
       </c>
       <c r="H9" s="15" t="n">
-        <v>81.63265306122449</v>
+        <v>72.44897959183675</v>
       </c>
       <c r="I9" s="15" t="n">
-        <v>18.36734693877551</v>
+        <v>27.55102040816326</v>
       </c>
       <c r="J9" s="15" t="n">
         <v>100</v>
@@ -4075,22 +4075,22 @@
         </is>
       </c>
       <c r="D10" s="15" t="n">
-        <v>0.1699668078287743</v>
+        <v>0.01525210837968782</v>
       </c>
       <c r="E10" s="15" t="n">
-        <v>25.51020408163265</v>
+        <v>12.24489795918367</v>
       </c>
       <c r="F10" s="15" t="n">
-        <v>48.97959183673469</v>
+        <v>40.81632653061224</v>
       </c>
       <c r="G10" s="15" t="n">
-        <v>74.48979591836735</v>
+        <v>53.06122448979592</v>
       </c>
       <c r="H10" s="15" t="n">
-        <v>74.48979591836735</v>
+        <v>53.06122448979592</v>
       </c>
       <c r="I10" s="15" t="n">
-        <v>25.51020408163265</v>
+        <v>46.93877551020408</v>
       </c>
       <c r="J10" s="15" t="n">
         <v>100</v>
@@ -4462,22 +4462,22 @@
         </is>
       </c>
       <c r="D19" s="15" t="n">
-        <v>0.1745722138487455</v>
+        <v>0.0495781508219536</v>
       </c>
       <c r="E19" s="15" t="n">
-        <v>4.081632653061225</v>
+        <v>10.20408163265306</v>
       </c>
       <c r="F19" s="15" t="n">
-        <v>63.26530612244898</v>
+        <v>43.87755102040816</v>
       </c>
       <c r="G19" s="15" t="n">
-        <v>67.3469387755102</v>
+        <v>54.08163265306123</v>
       </c>
       <c r="H19" s="15" t="n">
-        <v>67.34693877551021</v>
+        <v>54.08163265306122</v>
       </c>
       <c r="I19" s="15" t="n">
-        <v>32.6530612244898</v>
+        <v>45.91836734693878</v>
       </c>
       <c r="J19" s="15" t="n">
         <v>100</v>
@@ -4849,25 +4849,25 @@
         </is>
       </c>
       <c r="D28" s="15" t="n">
-        <v>0.1389564747228981</v>
+        <v>0.09841092835238363</v>
       </c>
       <c r="E28" s="15" t="n">
-        <v>34.69387755102041</v>
+        <v>38.77551020408163</v>
       </c>
       <c r="F28" s="15" t="n">
-        <v>42.85714285714285</v>
+        <v>36.73469387755102</v>
       </c>
       <c r="G28" s="15" t="n">
-        <v>77.55102040816327</v>
+        <v>75.51020408163265</v>
       </c>
       <c r="H28" s="15" t="n">
-        <v>77.55102040816325</v>
+        <v>75.51020408163265</v>
       </c>
       <c r="I28" s="15" t="n">
-        <v>22.44897959183674</v>
+        <v>24.48979591836735</v>
       </c>
       <c r="J28" s="15" t="n">
-        <v>99.99999999999999</v>
+        <v>100</v>
       </c>
       <c r="K28" s="14" t="inlineStr">
         <is>
@@ -5236,22 +5236,22 @@
         </is>
       </c>
       <c r="D37" s="15" t="n">
-        <v>0.07470147181338516</v>
+        <v>0.04499856692462023</v>
       </c>
       <c r="E37" s="15" t="n">
-        <v>30.61224489795918</v>
+        <v>40.81632653061224</v>
       </c>
       <c r="F37" s="15" t="n">
-        <v>47.95918367346938</v>
+        <v>32.6530612244898</v>
       </c>
       <c r="G37" s="15" t="n">
-        <v>78.57142857142857</v>
+        <v>73.46938775510205</v>
       </c>
       <c r="H37" s="15" t="n">
-        <v>78.57142857142857</v>
+        <v>73.46938775510205</v>
       </c>
       <c r="I37" s="15" t="n">
-        <v>21.42857142857143</v>
+        <v>26.53061224489796</v>
       </c>
       <c r="J37" s="15" t="n">
         <v>100</v>
@@ -5273,7 +5273,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A33"/>
+  <dimension ref="A1:A38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -5333,154 +5333,189 @@
     <row r="10">
       <c r="A10" s="17" t="inlineStr">
         <is>
-          <t>Weighted_Hazard = 0.35*Norm_Wind Gust + 0.35*Norm_Rainfall + 0.30*Norm_Storm Surge</t>
+          <t>Weighted_Hazard = w_wind*Norm_Wind Gust + w_rain*Norm_Rainfall + w_surge*Norm_Storm Surge</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="17" t="inlineStr">
         <is>
-          <t>Equivalent Excel columns: 0.35*H + 0.35*J + 0.30*L.</t>
+          <t>Equivalent Excel columns: w_wind*H + w_rain*J + w_surge*L.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17" t="inlineStr"/>
+      <c r="A12" s="16" t="inlineStr">
+        <is>
+          <t>Weights used for Midhili (see HAZARD_WEIGHTS in the script):</t>
+        </is>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>Forecast severity boundaries:</t>
+      <c r="A13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1dlt: w_wind=0.35, w_rain=0.35, w_surge=0.3</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="17" t="inlineStr">
         <is>
-          <t>Derived independently for each lead exactly as in the repository.</t>
+          <t xml:space="preserve">  2dlt: w_wind=0.35, w_rain=0.35, w_surge=0.3</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="17" t="inlineStr">
         <is>
-          <t>House: from Norm_Impact_House using Excel AG class labels.</t>
+          <t xml:space="preserve">  3dlt: w_wind=0.5, w_rain=0.5, w_surge=0.0</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>Agriculture: from Norm_Impact_fAPAR using Excel X class labels.</t>
+          <t>Weights differ by cyclone and by lead time and are set manually in HAZARD_WEIGHTS.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="17" t="inlineStr">
-        <is>
-          <t>Thresholds are rounded to 4 decimals before classification.</t>
-        </is>
-      </c>
+      <c r="A17" s="17" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="17" t="inlineStr">
-        <is>
-          <t>The same lead-specific sector boundary set is applied to Composite, Vulnerability-only and Hazard-only.</t>
+      <c r="A18" s="16" t="inlineStr">
+        <is>
+          <t>Forecast severity boundaries:</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="17" t="inlineStr"/>
+      <c r="A19" s="17" t="inlineStr">
+        <is>
+          <t>Derived independently for each lead exactly as in the repository.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
-        <is>
-          <t>DDM calibration:</t>
+      <c r="A20" s="17" t="inlineStr">
+        <is>
+          <t>House: from Norm_Impact_House using Excel AG class labels.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="17" t="inlineStr">
         <is>
-          <t>Zero = No Impact.</t>
+          <t>Agriculture: from Norm_Impact_fAPAR using Excel X class labels.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>Positive DDM values are exhaustively searched for Low/High cut pairs.</t>
+          <t>Thresholds are rounded to 4 decimals before classification.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
-          <t>For each candidate pair, QWK is calculated separately for 1dlt, 2dlt and 3dlt.</t>
+          <t>The same lead-specific sector boundary set is applied to Composite, Vulnerability-only and Hazard-only.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="inlineStr">
-        <is>
-          <t>The mean of the three Kappas is maximized.</t>
-        </is>
-      </c>
+      <c r="A24" s="17" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="17" t="inlineStr">
-        <is>
-          <t>The selected Low/High pair is then fixed for all three leads for that predictor and damage variable.</t>
+      <c r="A25" s="16" t="inlineStr">
+        <is>
+          <t>DDM calibration:</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="17" t="inlineStr">
         <is>
-          <t>The maximum positive observed DDM value is excluded as a High cut so that the High class remains populated.</t>
+          <t>Zero = No Impact.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="17" t="inlineStr"/>
+      <c r="A27" s="17" t="inlineStr">
+        <is>
+          <t>Positive DDM values are exhaustively searched for Low/High cut pairs.</t>
+        </is>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
-        <is>
-          <t>Agreement table:</t>
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>For each candidate pair, QWK is calculated separately for 1dlt, 2dlt and 3dlt.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="17" t="inlineStr">
         <is>
-          <t>Exact = difference of 0 classes.</t>
+          <t>The mean of the three Kappas is maximized.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="17" t="inlineStr">
         <is>
-          <t>Adjacent = difference of exactly 1 class.</t>
+          <t>The selected Low/High pair is then fixed for all three leads for that predictor and damage variable.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="17" t="inlineStr">
         <is>
+          <t>The maximum positive observed DDM value is excluded as a High cut so that the High class remains populated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Agreement table:</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="17" t="inlineStr">
+        <is>
+          <t>Exact = difference of 0 classes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="17" t="inlineStr">
+        <is>
+          <t>Adjacent = difference of exactly 1 class.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="17" t="inlineStr">
+        <is>
           <t>Off-Cat. = difference of 2 or more classes.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
         <is>
           <t>Exact + Adjacent + Off-Cat. = 100%.</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="17" t="inlineStr">
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Repository Within-1 % = Exact % + Adjacent %.</t>
         </is>

</xml_diff>